<commit_message>
Project plan: remove 'chosen by Tony' from notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CBrkjaB9ndxyBKBoLJhs7C
</commit_message>
<xml_diff>
--- a/docs/Team_B_Project_Plan.xlsx
+++ b/docs/Team_B_Project_Plan.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -475,6 +473,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -1243,24 +1242,25 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Work starts Mon Oct 12, 2026; final presentation Thu Dec 10, 2026 (chosen by Tony).</t>
+          <t>Work starts Mon Oct 12, 2026; final presentation Thu Dec 10, 2026.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The app connects to the SQL Server database through a back-end API before the presentation (chosen by Tony).</t>
+          <t>The app connects to the SQL Server database through a back-end API before the presentation.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Database owner: Carlos. Back end and integration: Tony and Carlos. Jared and Rob: page polish, testing, test plans (chosen by Tony).</t>
+          <t>Database owner: Carlos. Back end and integration: Tony and Carlos. Jared and Rob: page polish, testing, test plans.</t>
         </is>
       </c>
     </row>

</xml_diff>